<commit_message>
Committing update Booking module
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDataAPI.xlsx
+++ b/src/test/resources/TestDataAPI.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bec74d40107829ab/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="8_{7259C6C2-5F91-4927-863F-CC7DDADB99D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E221A26E-3F6E-41B8-B9DE-29F89ED3D2D6}"/>
+  <xr:revisionPtr revIDLastSave="121" documentId="8_{7259C6C2-5F91-4927-863F-CC7DDADB99D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06A0D1DC-BD75-48C5-A4BE-4632CAA43E0C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{3B802E28-E2CE-4EED-8F88-E5E4A5BE7189}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{3B802E28-E2CE-4EED-8F88-E5E4A5BE7189}"/>
   </bookViews>
   <sheets>
     <sheet name="Auth" sheetId="1" r:id="rId1"/>
     <sheet name="CreateBooking" sheetId="2" r:id="rId2"/>
     <sheet name="GetBooking" sheetId="3" r:id="rId3"/>
+    <sheet name="UpdateBooking" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="40">
   <si>
     <t>TestCase</t>
   </si>
@@ -137,6 +138,27 @@
   </si>
   <si>
     <t>Additionalneeds</t>
+  </si>
+  <si>
+    <t>TC25</t>
+  </si>
+  <si>
+    <t>Dinner</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>TC26</t>
+  </si>
+  <si>
+    <t>TC27</t>
+  </si>
+  <si>
+    <t>TC28</t>
+  </si>
+  <si>
+    <t>lkaf23</t>
   </si>
 </sst>
 </file>
@@ -845,4 +867,120 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B96E129-E6F9-40FB-A91E-A2713B680F14}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2">
+        <v>571</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2">
+        <v>3000</v>
+      </c>
+      <c r="E2" s="2">
+        <v>46259</v>
+      </c>
+      <c r="F2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3">
+        <v>571</v>
+      </c>
+      <c r="C3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3">
+        <v>3000</v>
+      </c>
+      <c r="E3" s="2">
+        <v>46259</v>
+      </c>
+      <c r="F3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4">
+        <v>571</v>
+      </c>
+      <c r="C4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4">
+        <v>3000</v>
+      </c>
+      <c r="E4" s="2">
+        <v>46259</v>
+      </c>
+      <c r="F4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5">
+        <v>3000</v>
+      </c>
+      <c r="E5" s="2">
+        <v>46259</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>